<commit_message>
conectado con IA NO TOCAR!!!
</commit_message>
<xml_diff>
--- a/db/BASE_DE_DATOS_GENERAL.xlsx
+++ b/db/BASE_DE_DATOS_GENERAL.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AC6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,7 +407,7 @@
         <v>Tipo_unidad</v>
       </c>
       <c r="C1" t="str">
-        <v>Antiguedad_años</v>
+        <v>Antiguedad_anos</v>
       </c>
       <c r="D1" t="str">
         <v>Tipo_operacion</v>
@@ -483,6 +483,9 @@
       </c>
       <c r="AB1" t="str">
         <v>comentario_general</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>consumo_normal</v>
       </c>
     </row>
     <row r="2">
@@ -642,13 +645,13 @@
         <v>20</v>
       </c>
       <c r="Z3" t="str" xml:space="preserve">
-        <v xml:space="preserve">[_x000d__x000d_
-  {_x000d__x000d_
-    "nombre_mantenimiento": "Afinación mayor y cambio de aceite",_x000d__x000d_
-    "fecha_solicitud": "2025-11-10",_x000d__x000d_
-    "concluido": true,_x000d__x000d_
-    "fecha_realizacion": "2025-11-12"_x000d__x000d_
-  }_x000d__x000d_
+        <v xml:space="preserve">[_x000d__x000d__x000d_
+  {_x000d__x000d__x000d_
+    "nombre_mantenimiento": "Afinación mayor y cambio de aceite",_x000d__x000d__x000d_
+    "fecha_solicitud": "2025-11-10",_x000d__x000d__x000d_
+    "concluido": true,_x000d__x000d__x000d_
+    "fecha_realizacion": "2025-11-12"_x000d__x000d__x000d_
+  }_x000d__x000d__x000d_
 ]</v>
       </c>
     </row>
@@ -761,9 +764,92 @@
         <v>nopiti, todo esta bien</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>123456</v>
+      </c>
+      <c r="B6" t="str">
+        <v>tractocamion</v>
+      </c>
+      <c r="C6" t="str">
+        <v>50</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Urbano</v>
+      </c>
+      <c r="E6" t="str">
+        <v>10000</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Malo</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2</v>
+      </c>
+      <c r="H6" t="str">
+        <v>160000</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="K6" t="str">
+        <v>No</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Regular</v>
+      </c>
+      <c r="P6" t="str">
+        <v>20</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>15000</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Bajo</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Medio</v>
+      </c>
+      <c r="T6" t="str">
+        <v>Alto</v>
+      </c>
+      <c r="U6" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="V6" t="str">
+        <v>Diagnóstico: Falla en tren motriz, motor y suspensión trasera. Requiere atención inmediata.</v>
+      </c>
+      <c r="W6" t="str">
+        <v>URGENTE</v>
+      </c>
+      <c r="X6">
+        <v>95</v>
+      </c>
+      <c r="Y6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AA6" t="str">
+        <v>Recepción</v>
+      </c>
+      <c r="AB6" t="str">
+        <v>Qué tal jefe, le reporto que el camión me viene temblando muchísimo de la parte de atrás, como en el eje. Además, en las subidas siento que no jala, le piso a fondo y pierde mucha fuerza. Por si fuera poco, se me prendió fijo el foquito amarillo del motor en el tablero. Ahorita lo traigo despacio para no quedarme tirado, pero sí urge que el mecánico lo revise llegando al patio porque es peligroso.</v>
+      </c>
+      <c r="AC6" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
no le muevas NADA
</commit_message>
<xml_diff>
--- a/db/BASE_DE_DATOS_GENERAL.xlsx
+++ b/db/BASE_DE_DATOS_GENERAL.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC6"/>
+  <dimension ref="A1:AC12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -645,13 +645,13 @@
         <v>20</v>
       </c>
       <c r="Z3" t="str" xml:space="preserve">
-        <v xml:space="preserve">[_x000d__x000d__x000d_
-  {_x000d__x000d__x000d_
-    "nombre_mantenimiento": "Afinación mayor y cambio de aceite",_x000d__x000d__x000d_
-    "fecha_solicitud": "2025-11-10",_x000d__x000d__x000d_
-    "concluido": true,_x000d__x000d__x000d_
-    "fecha_realizacion": "2025-11-12"_x000d__x000d__x000d_
-  }_x000d__x000d__x000d_
+        <v xml:space="preserve">[_x000d__x000d__x000d__x000d_
+  {_x000d__x000d__x000d__x000d_
+    "nombre_mantenimiento": "Afinación mayor y cambio de aceite",_x000d__x000d__x000d__x000d_
+    "fecha_solicitud": "2025-11-10",_x000d__x000d__x000d__x000d_
+    "concluido": true,_x000d__x000d__x000d__x000d_
+    "fecha_realizacion": "2025-11-12"_x000d__x000d__x000d__x000d_
+  }_x000d__x000d__x000d__x000d_
 ]</v>
       </c>
     </row>
@@ -847,9 +847,201 @@
         <v>No</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>0000</v>
+      </c>
+      <c r="B7" t="str">
+        <v>hola</v>
+      </c>
+      <c r="C7" t="str">
+        <v>1</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Carretera</v>
+      </c>
+      <c r="E7" t="str">
+        <v>10</v>
+      </c>
+      <c r="V7" t="str">
+        <v>Unidad en estado estable. Se recomienda monitoreo preventivo.</v>
+      </c>
+      <c r="W7" t="str">
+        <v>ESTABLE</v>
+      </c>
+      <c r="X7">
+        <v>10</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>111111</v>
+      </c>
+      <c r="B8" t="str">
+        <v>tracto</v>
+      </c>
+      <c r="C8" t="str">
+        <v>50</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Mixto</v>
+      </c>
+      <c r="E8" t="str">
+        <v>20</v>
+      </c>
+      <c r="V8" t="str">
+        <v>Revisar mangueras de refrigerante y origen de zumbido. Corregir antes de generar fuga.</v>
+      </c>
+      <c r="W8" t="str">
+        <v>PREVENTIVO</v>
+      </c>
+      <c r="X8">
+        <v>70</v>
+      </c>
+      <c r="Y8" t="str">
+        <v>150</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>"Hola, entregando unidad. En general el camión anduvo bien en el trayecto, pero cuando me paré a comer y revisé por abajo, noté que dejó unas gotitas de líquido fresco, creo que viene de alguna manguera reseca. También le noto un zumbidito leve cuando acelero, no prende nada en el tablero, pero mejor que le echen un ojo rápido en el taller antes de que se reviente algo y se haga una fuga más grande."</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>222222</v>
+      </c>
+      <c r="B9" t="str">
+        <v>mercedes</v>
+      </c>
+      <c r="C9" t="str">
+        <v>20</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Mixto</v>
+      </c>
+      <c r="E9" t="str">
+        <v>10</v>
+      </c>
+      <c r="V9" t="str">
+        <v>Revisar fugas de líquido y zumbido de aceleración. Posible desgaste de mangueras o componentes del motor.</v>
+      </c>
+      <c r="W9" t="str">
+        <v>PREVENTIVO</v>
+      </c>
+      <c r="X9">
+        <v>70</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>800</v>
+      </c>
+      <c r="AB9" t="str">
+        <v>"Hola, entregando unidad. En general el camión anduvo bien en el trayecto, pero cuando me paré a comer y revisé por abajo, noté que dejó unas gotitas de líquido fresco, creo que viene de alguna manguera reseca. También le noto un zumbidito leve cuando acelero, no prende nada en el tablero, pero mejor que le echen un ojo rápido en el taller antes de que se reviente algo y se haga una fuga más grande."</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>3333333</v>
+      </c>
+      <c r="B10" t="str">
+        <v>emerece</v>
+      </c>
+      <c r="C10" t="str">
+        <v>50</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Mixto</v>
+      </c>
+      <c r="E10" t="str">
+        <v>8000</v>
+      </c>
+      <c r="V10" t="str">
+        <v>Inspeccionar mangueras de líquido fresco y evaluar posible causa del zumbido al acelerar.</v>
+      </c>
+      <c r="W10" t="str">
+        <v>PREVENTIVO</v>
+      </c>
+      <c r="X10">
+        <v>65</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>10</v>
+      </c>
+      <c r="AB10" t="str">
+        <v>"Hola, entregando unidad. En general el camión anduvo bien en el trayecto, pero cuando me paré a comer y revisé por abajo, noté que dejó unas gotitas de líquido fresco, creo que viene de alguna manguera reseca. También le noto un zumbidito leve cuando acelero, no prende nada en el tablero, pero mejor que le echen un ojo rápido en el taller antes de que se reviente algo y se haga una fuga más grande."</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>444444</v>
+      </c>
+      <c r="B11" t="str">
+        <v>sdf</v>
+      </c>
+      <c r="C11" t="str">
+        <v>4</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Urbano</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2</v>
+      </c>
+      <c r="V11" t="str">
+        <v>Revisar mangueras de refrigerante y sistema de admisión por posible fuga y zumbido.</v>
+      </c>
+      <c r="W11" t="str">
+        <v>PREVENTIVO</v>
+      </c>
+      <c r="X11">
+        <v>65</v>
+      </c>
+      <c r="Y11" t="str">
+        <v>1</v>
+      </c>
+      <c r="AB11" t="str">
+        <v>"Hola, entregando unidad. En general el camión anduvo bien en el trayecto, pero cuando me paré a comer y revisé por abajo, noté que dejó unas gotitas de líquido fresco, creo que viene de alguna manguera reseca. También le noto un zumbidito leve cuando acelero, no prende nada en el tablero, pero mejor que le echen un ojo rápido en el taller antes de que se reviente algo y se haga una fuga más grande."</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>888888</v>
+      </c>
+      <c r="B12" t="str">
+        <v>dgf</v>
+      </c>
+      <c r="C12" t="str">
+        <v>150</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Urbano</v>
+      </c>
+      <c r="E12" t="str">
+        <v>1</v>
+      </c>
+      <c r="V12" t="str">
+        <v>Revisar mangueras de refrigeración y sistema de aceleración. Inspeccionar posibles fugas.</v>
+      </c>
+      <c r="W12" t="str">
+        <v>PREVENTIVO</v>
+      </c>
+      <c r="X12">
+        <v>75</v>
+      </c>
+      <c r="Y12" t="str">
+        <v>1</v>
+      </c>
+      <c r="Z12" t="str">
+        <v>[{"nombre_mantenimiento":"Reemplazo de banda de distribución","fecha_solicitud":"2026-04-05","concluido":false,"fecha_realizacion":""},{"nombre_mantenimiento":"Inspección y sellado de fugas en mangueras de presión","fecha_solicitud":"2026-04-05","concluido":false,"fecha_realizacion":""},{"nombre_mantenimiento":"Cambio de aceite y filtros de motor","fecha_solicitud":"2026-04-06","concluido":true,"fecha_realizacion":"2026-04-08"}]</v>
+      </c>
+      <c r="AB12" t="str">
+        <v>"Hola, entregando unidad. En general el camión anduvo bien en el trayecto, pero cuando me paré a comer y revisé por abajo, noté que dejó unas gotitas de líquido fresco, creo que viene de alguna manguera reseca. También le noto un zumbidito leve cuando acelero, no prende nada en el tablero, pero mejor que le echen un ojo rápido en el taller antes de que se reviente algo y se haga una fuga más grande."</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>